<commit_message>
Re-ran everything, fixing a few minor isses with glmer
</commit_message>
<xml_diff>
--- a/Output/mainresults.xlsx
+++ b/Output/mainresults.xlsx
@@ -418,22 +418,22 @@
         </is>
       </c>
       <c r="D2">
-        <v>0.01987143426751635</v>
+        <v>0.01987123247152484</v>
       </c>
       <c r="E2">
-        <v>0.004961787724162165</v>
+        <v>0.004961789114915679</v>
       </c>
       <c r="F2">
-        <v>4.004894076937117</v>
+        <v>4.004852284388658</v>
       </c>
       <c r="G2">
-        <v>6.204527671571261E-05</v>
+        <v>6.205624685957044E-05</v>
       </c>
       <c r="H2">
-        <v>0.01014650902922555</v>
+        <v>0.01014630450740724</v>
       </c>
       <c r="I2">
-        <v>0.02959635950580716</v>
+        <v>0.02959616043564244</v>
       </c>
     </row>
     <row r="3">
@@ -453,22 +453,22 @@
         </is>
       </c>
       <c r="D3">
-        <v>0.0001832961695471341</v>
+        <v>0.0001832962116385026</v>
       </c>
       <c r="E3">
-        <v>0.007262161922928861</v>
+        <v>0.007262161930453457</v>
       </c>
       <c r="F3">
-        <v>0.02523989019969552</v>
+        <v>0.02523989596952672</v>
       </c>
       <c r="G3">
-        <v>0.9798636193031247</v>
+        <v>0.9798636147009315</v>
       </c>
       <c r="H3">
-        <v>-0.01405027964929157</v>
+        <v>-0.01405027962194814</v>
       </c>
       <c r="I3">
-        <v>0.01441687198838584</v>
+        <v>0.01441687204522515</v>
       </c>
     </row>
     <row r="4">
@@ -488,22 +488,22 @@
         </is>
       </c>
       <c r="D4">
-        <v>0.01798467081903042</v>
+        <v>0.01798592711810813</v>
       </c>
       <c r="E4">
-        <v>0.0071138277807318</v>
+        <v>0.00711382540231625</v>
       </c>
       <c r="F4">
-        <v>2.528128508781574</v>
+        <v>2.528305953678866</v>
       </c>
       <c r="G4">
-        <v>0.01146723701557349</v>
+        <v>0.01146144240894549</v>
       </c>
       <c r="H4">
-        <v>0.004041824576575596</v>
+        <v>0.004043085537262124</v>
       </c>
       <c r="I4">
-        <v>0.03192751706148525</v>
+        <v>0.03192876869895413</v>
       </c>
     </row>
     <row r="5">
@@ -523,22 +523,22 @@
         </is>
       </c>
       <c r="D5">
-        <v>0.002720766972376285</v>
+        <v>0.00269049014985419</v>
       </c>
       <c r="E5">
-        <v>0.008423904286238954</v>
+        <v>0.008414857175553568</v>
       </c>
       <c r="F5">
-        <v>0.3229817053858092</v>
+        <v>0.3197309346699871</v>
       </c>
       <c r="G5">
-        <v>0.746709097169707</v>
+        <v>0.7491723072792718</v>
       </c>
       <c r="H5">
-        <v>-0.01378978203786465</v>
+        <v>-0.01380232684927924</v>
       </c>
       <c r="I5">
-        <v>0.01923131598261722</v>
+        <v>0.01918330714898762</v>
       </c>
     </row>
     <row r="6">
@@ -558,22 +558,22 @@
         </is>
       </c>
       <c r="D6">
-        <v>0.01623324829873208</v>
+        <v>0.01396321459412943</v>
       </c>
       <c r="E6">
-        <v>0.007447953647820331</v>
+        <v>0.007429933057411854</v>
       </c>
       <c r="F6">
-        <v>2.179558180183196</v>
+        <v>1.879319031037594</v>
       </c>
       <c r="G6">
-        <v>0.02929022758439538</v>
+        <v>0.06020094465454619</v>
       </c>
       <c r="H6">
-        <v>0.001635527390480515</v>
+        <v>-0.0005991866059413663</v>
       </c>
       <c r="I6">
-        <v>0.03083096920698365</v>
+        <v>0.02852561579420024</v>
       </c>
     </row>
     <row r="7">
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="D7">
-        <v>0.01333478743963215</v>
+        <v>0.01333967370819499</v>
       </c>
       <c r="E7">
-        <v>0.01790489929032319</v>
+        <v>0.01789403879291838</v>
       </c>
       <c r="F7">
-        <v>0.7447563498354336</v>
+        <v>0.7454814344917037</v>
       </c>
       <c r="G7">
-        <v>0.4564190271047672</v>
+        <v>0.4559807304517166</v>
       </c>
       <c r="H7">
-        <v>-0.02175817031621808</v>
+        <v>-0.02173199786388762</v>
       </c>
       <c r="I7">
-        <v>0.04842774519548237</v>
+        <v>0.0484113452802776</v>
       </c>
     </row>
     <row r="8">
@@ -628,22 +628,22 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.02364277775111993</v>
+        <v>0.02364309104058191</v>
       </c>
       <c r="E8">
-        <v>0.01501968953997905</v>
+        <v>0.01501976188292623</v>
       </c>
       <c r="F8">
-        <v>1.5741189382236</v>
+        <v>1.574132214935996</v>
       </c>
       <c r="G8">
-        <v>0.1154599550681725</v>
+        <v>0.1154568862745276</v>
       </c>
       <c r="H8">
-        <v>-0.005795272806211973</v>
+        <v>-0.005795101306320997</v>
       </c>
       <c r="I8">
-        <v>0.05308082830845184</v>
+        <v>0.05308128338748482</v>
       </c>
     </row>
     <row r="9">
@@ -663,22 +663,22 @@
         </is>
       </c>
       <c r="D9">
-        <v>-0.006886807422543868</v>
+        <v>-0.007795905394822687</v>
       </c>
       <c r="E9">
-        <v>0.01799047069112808</v>
+        <v>0.01798650494647843</v>
       </c>
       <c r="F9">
-        <v>-0.3828030706244981</v>
+        <v>-0.4334308092662017</v>
       </c>
       <c r="G9">
-        <v>0.7018657845763321</v>
+        <v>0.6647018220572505</v>
       </c>
       <c r="H9">
-        <v>-0.04214748204207832</v>
+        <v>-0.04304880729767194</v>
       </c>
       <c r="I9">
-        <v>0.02837386719699058</v>
+        <v>0.02745699650802657</v>
       </c>
     </row>
     <row r="10">
@@ -698,22 +698,22 @@
         </is>
       </c>
       <c r="D10">
-        <v>-0.01956303578930273</v>
+        <v>-0.01956338868373303</v>
       </c>
       <c r="E10">
-        <v>0.01788427029661514</v>
+        <v>0.01788409341440013</v>
       </c>
       <c r="F10">
-        <v>-1.09386826886671</v>
+        <v>-1.093898820053173</v>
       </c>
       <c r="G10">
-        <v>0.2740127572276837</v>
+        <v>0.2739993563317618</v>
       </c>
       <c r="H10">
-        <v>-0.05461556146044787</v>
+        <v>-0.05461556767210723</v>
       </c>
       <c r="I10">
-        <v>0.0154894898818424</v>
+        <v>0.01548879030464118</v>
       </c>
     </row>
     <row r="11">
@@ -733,22 +733,22 @@
         </is>
       </c>
       <c r="D11">
-        <v>0.04947352423294215</v>
+        <v>0.04957281677095193</v>
       </c>
       <c r="E11">
-        <v>0.006645543852715086</v>
+        <v>0.006645704763297719</v>
       </c>
       <c r="F11">
-        <v>7.44461632176716</v>
+        <v>7.459376926391325</v>
       </c>
       <c r="G11">
-        <v>9.722657216075414E-14</v>
+        <v>8.693258761586841E-14</v>
       </c>
       <c r="H11">
-        <v>0.03644849762393903</v>
+        <v>0.03654747478300212</v>
       </c>
       <c r="I11">
-        <v>0.06249855084194527</v>
+        <v>0.06259815875890173</v>
       </c>
     </row>
     <row r="12">
@@ -768,22 +768,22 @@
         </is>
       </c>
       <c r="D12">
-        <v>0.04586855848303279</v>
+        <v>0.0458685584085329</v>
       </c>
       <c r="E12">
-        <v>0.009834807506769197</v>
+        <v>0.009834807510044242</v>
       </c>
       <c r="F12">
-        <v>4.66389997480499</v>
+        <v>4.663899965676761</v>
       </c>
       <c r="G12">
-        <v>3.102722380556536E-06</v>
+        <v>3.102722518260945E-06</v>
       </c>
       <c r="H12">
-        <v>0.026592689974881</v>
+        <v>0.02659268989396214</v>
       </c>
       <c r="I12">
-        <v>0.06514442699118458</v>
+        <v>0.06514442692310365</v>
       </c>
     </row>
     <row r="13">
@@ -803,22 +803,22 @@
         </is>
       </c>
       <c r="D13">
-        <v>0.06126268708049752</v>
+        <v>0.06371999230213674</v>
       </c>
       <c r="E13">
-        <v>0.009033438663248823</v>
+        <v>0.009036249755118058</v>
       </c>
       <c r="F13">
-        <v>6.78176820192907</v>
+        <v>7.051597070570814</v>
       </c>
       <c r="G13">
-        <v>1.187138407869338E-11</v>
+        <v>1.768757683192757E-12</v>
       </c>
       <c r="H13">
-        <v>0.04355747264397818</v>
+        <v>0.04600926822679646</v>
       </c>
       <c r="I13">
-        <v>0.07896790151701685</v>
+        <v>0.08143071637747701</v>
       </c>
     </row>
     <row r="14">
@@ -838,22 +838,22 @@
         </is>
       </c>
       <c r="D14">
-        <v>0.03977016629572373</v>
+        <v>0.0397701663017692</v>
       </c>
       <c r="E14">
-        <v>0.01312045464117798</v>
+        <v>0.01312030399786391</v>
       </c>
       <c r="F14">
-        <v>3.031157637701577</v>
+        <v>3.031192440986436</v>
       </c>
       <c r="G14">
-        <v>0.002436180226870007</v>
+        <v>0.002435899420700805</v>
       </c>
       <c r="H14">
-        <v>0.0140545477382235</v>
+        <v>0.01405484299973906</v>
       </c>
       <c r="I14">
-        <v>0.06548578485322396</v>
+        <v>0.06548548960379934</v>
       </c>
     </row>
     <row r="15">
@@ -873,22 +873,22 @@
         </is>
       </c>
       <c r="D15">
-        <v>0.03984602158473804</v>
+        <v>0.03984590650618706</v>
       </c>
       <c r="E15">
-        <v>0.01232359588857734</v>
+        <v>0.01232345437728853</v>
       </c>
       <c r="F15">
-        <v>3.233311279029448</v>
+        <v>3.233339069248387</v>
       </c>
       <c r="G15">
-        <v>0.001223641535237426</v>
+        <v>0.001223522496113945</v>
       </c>
       <c r="H15">
-        <v>0.01569221748310058</v>
+        <v>0.01569237976157907</v>
       </c>
       <c r="I15">
-        <v>0.06399982568637549</v>
+        <v>0.06399943325079506</v>
       </c>
     </row>
     <row r="16">
@@ -908,22 +908,22 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.05244259081769893</v>
+        <v>0.09897436377220174</v>
       </c>
       <c r="E16">
-        <v>9.226942806137777E-05</v>
+        <v>0.02076485433562381</v>
       </c>
       <c r="F16">
-        <v>568.3636706061951</v>
+        <v>4.766436699842537</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>1.875126047700802E-06</v>
       </c>
       <c r="H16">
-        <v>0.05226174606182452</v>
+        <v>0.0582759971301587</v>
       </c>
       <c r="I16">
-        <v>0.05262343557357334</v>
+        <v>0.1396727304142448</v>
       </c>
     </row>
     <row r="17">
@@ -943,22 +943,22 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.1047352533767841</v>
+        <v>0.1044140955199383</v>
       </c>
       <c r="E17">
-        <v>0.01937877648231309</v>
+        <v>0.01937893765513618</v>
       </c>
       <c r="F17">
-        <v>5.404637050867245</v>
+        <v>5.388019579714393</v>
       </c>
       <c r="G17">
-        <v>6.493975409178787E-08</v>
+        <v>7.12382931198159E-08</v>
       </c>
       <c r="H17">
-        <v>0.06675354940699868</v>
+        <v>0.06643207565722428</v>
       </c>
       <c r="I17">
-        <v>0.1427169573465696</v>
+        <v>0.1423961153826523</v>
       </c>
     </row>
     <row r="18">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.05193726163737072</v>
+        <v>0.05193697620010032</v>
       </c>
       <c r="E18">
-        <v>0.02325225627984554</v>
+        <v>0.02325230617619353</v>
       </c>
       <c r="F18">
-        <v>2.233643953184389</v>
+        <v>2.233626884428139</v>
       </c>
       <c r="G18">
-        <v>0.0255065094659875</v>
+        <v>0.02550763346708477</v>
       </c>
       <c r="H18">
-        <v>0.006363676769578164</v>
+        <v>0.006363293537262761</v>
       </c>
       <c r="I18">
-        <v>0.09751084650516328</v>
+        <v>0.09751065886293789</v>
       </c>
     </row>
     <row r="19">
@@ -1013,22 +1013,22 @@
         </is>
       </c>
       <c r="D19">
-        <v>0.06480183153932956</v>
+        <v>0.06480057971898644</v>
       </c>
       <c r="E19">
-        <v>0.02305151583207117</v>
+        <v>0.02305143151101756</v>
       </c>
       <c r="F19">
-        <v>2.811174415227475</v>
+        <v>2.811130392835457</v>
       </c>
       <c r="G19">
-        <v>0.004936102005392109</v>
+        <v>0.004936777451532664</v>
       </c>
       <c r="H19">
-        <v>0.01962169071941523</v>
+        <v>0.01962060416530031</v>
       </c>
       <c r="I19">
-        <v>0.1099819723592439</v>
+        <v>0.1099805552726726</v>
       </c>
     </row>
     <row r="20">
@@ -1048,22 +1048,22 @@
         </is>
       </c>
       <c r="D20">
-        <v>0.0050118114917662</v>
+        <v>0.005011857513695142</v>
       </c>
       <c r="E20">
-        <v>0.003229747794481636</v>
+        <v>0.00322974773983021</v>
       </c>
       <c r="F20">
-        <v>1.551765589972507</v>
+        <v>1.551779865618427</v>
       </c>
       <c r="G20">
-        <v>0.1207183221815232</v>
+        <v>0.1207149051768156</v>
       </c>
       <c r="H20">
-        <v>-0.001318377864565477</v>
+        <v>-0.001318331735521709</v>
       </c>
       <c r="I20">
-        <v>0.01134200084809788</v>
+        <v>0.01134204676291199</v>
       </c>
     </row>
     <row r="21">
@@ -1083,22 +1083,22 @@
         </is>
       </c>
       <c r="D21">
-        <v>0.004459276853191458</v>
+        <v>0.004510123080274954</v>
       </c>
       <c r="E21">
-        <v>0.004538491916662724</v>
+        <v>0.004540559459718427</v>
       </c>
       <c r="F21">
-        <v>0.9825459503011487</v>
+        <v>0.9932967776959007</v>
       </c>
       <c r="G21">
-        <v>0.3258309571033339</v>
+        <v>0.3205653474128138</v>
       </c>
       <c r="H21">
-        <v>-0.00443600384759364</v>
+        <v>-0.004389209930435807</v>
       </c>
       <c r="I21">
-        <v>0.01335455755397656</v>
+        <v>0.01340945609098572</v>
       </c>
     </row>
     <row r="22">
@@ -1118,22 +1118,22 @@
         </is>
       </c>
       <c r="D22">
-        <v>0.001050349619761949</v>
+        <v>0.001040739083847438</v>
       </c>
       <c r="E22">
-        <v>0.004545355113149121</v>
+        <v>0.004544729136515466</v>
       </c>
       <c r="F22">
-        <v>0.2310819712905212</v>
+        <v>0.2289991444122439</v>
       </c>
       <c r="G22">
-        <v>0.8172511209337914</v>
+        <v>0.8188695811187787</v>
       </c>
       <c r="H22">
-        <v>-0.007858382698955309</v>
+        <v>-0.007866766343212692</v>
       </c>
       <c r="I22">
-        <v>0.009959081938479207</v>
+        <v>0.009948244510907568</v>
       </c>
     </row>
     <row r="23">
@@ -1153,22 +1153,22 @@
         </is>
       </c>
       <c r="D23">
-        <v>0.0006825039839203173</v>
+        <v>0.005145024064844539</v>
       </c>
       <c r="E23">
-        <v>4.443660587626631E-05</v>
+        <v>0.003526476377567667</v>
       </c>
       <c r="F23">
-        <v>15.35904847955195</v>
+        <v>1.458970233736045</v>
       </c>
       <c r="G23">
-        <v>3.080628498892604E-53</v>
+        <v>0.144573300570708</v>
       </c>
       <c r="H23">
-        <v>0.0005954098368076344</v>
+        <v>-0.001766742627519359</v>
       </c>
       <c r="I23">
-        <v>0.0007695981310330001</v>
+        <v>0.01205679075720844</v>
       </c>
     </row>
     <row r="24">
@@ -1188,22 +1188,22 @@
         </is>
       </c>
       <c r="D24">
-        <v>0.00336897099845952</v>
+        <v>0.003369023835965095</v>
       </c>
       <c r="E24">
-        <v>0.003916198991833251</v>
+        <v>0.003916263381891891</v>
       </c>
       <c r="F24">
-        <v>0.8602655292759873</v>
+        <v>0.8602648768575845</v>
       </c>
       <c r="G24">
-        <v>0.3896426897889415</v>
+        <v>0.3896430493437474</v>
       </c>
       <c r="H24">
-        <v>-0.00430663798182572</v>
+        <v>-0.004306711346516041</v>
       </c>
       <c r="I24">
-        <v>0.01104457997874476</v>
+        <v>0.01104475901844623</v>
       </c>
     </row>
     <row r="25">
@@ -1223,22 +1223,22 @@
         </is>
       </c>
       <c r="D25">
-        <v>0.001227185205059252</v>
+        <v>0.001227185380792179</v>
       </c>
       <c r="E25">
-        <v>0.01089481814254631</v>
+        <v>0.01089471460942329</v>
       </c>
       <c r="F25">
-        <v>0.1126393473487055</v>
+        <v>0.1126404338972529</v>
       </c>
       <c r="G25">
-        <v>0.9103164888707682</v>
+        <v>0.9103156274128085</v>
       </c>
       <c r="H25">
-        <v>-0.02012626597244507</v>
+        <v>-0.02012606287551982</v>
       </c>
       <c r="I25">
-        <v>0.02258063638256358</v>
+        <v>0.02258043363710418</v>
       </c>
     </row>
     <row r="26">
@@ -1258,22 +1258,22 @@
         </is>
       </c>
       <c r="D26">
-        <v>0.01915780019998702</v>
+        <v>0.0191571266577937</v>
       </c>
       <c r="E26">
-        <v>0.009506307602736097</v>
+        <v>0.00950624639709889</v>
       </c>
       <c r="F26">
-        <v>2.015272490706385</v>
+        <v>2.015214613376743</v>
       </c>
       <c r="G26">
-        <v>0.04387610566430804</v>
+        <v>0.04388216700568755</v>
       </c>
       <c r="H26">
-        <v>0.0005257796726649729</v>
+        <v>0.0005252260913162325</v>
       </c>
       <c r="I26">
-        <v>0.03778982072730906</v>
+        <v>0.03778902722427117</v>
       </c>
     </row>
     <row r="27">
@@ -1293,22 +1293,22 @@
         </is>
       </c>
       <c r="D27">
-        <v>0.01383760620407962</v>
+        <v>0.01381522916158572</v>
       </c>
       <c r="E27">
-        <v>0.01658081415119263</v>
+        <v>0.01658058259384839</v>
       </c>
       <c r="F27">
-        <v>0.8345552925146507</v>
+        <v>0.8332173542992001</v>
       </c>
       <c r="G27">
-        <v>0.4039681431592572</v>
+        <v>0.4047221568213121</v>
       </c>
       <c r="H27">
-        <v>-0.01866019236660998</v>
+        <v>-0.01868211556504883</v>
       </c>
       <c r="I27">
-        <v>0.04633540477476923</v>
+        <v>0.04631257388822027</v>
       </c>
     </row>
     <row r="28">
@@ -1328,22 +1328,22 @@
         </is>
       </c>
       <c r="D28">
-        <v>-0.02875493208931094</v>
+        <v>-0.02855311784491485</v>
       </c>
       <c r="E28">
-        <v>0.01623552039303771</v>
+        <v>0.01623058298363427</v>
       </c>
       <c r="F28">
-        <v>-1.771112437002138</v>
+        <v>-1.759217020960105</v>
       </c>
       <c r="G28">
-        <v>0.07654200624551558</v>
+        <v>0.07854065430328687</v>
       </c>
       <c r="H28">
-        <v>-0.06057596732993044</v>
+        <v>-0.06036447594092667</v>
       </c>
       <c r="I28">
-        <v>0.003066103151308553</v>
+        <v>0.003258240251096972</v>
       </c>
     </row>
   </sheetData>

</xml_diff>